<commit_message>
docs: corregir id 89703 en evidencia TC-NOTIF-001 matriz
Co-authored-by: JFCandia-Digital <JFCandia-Digital@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/api-v3.5/matriz_api_notificacion_DocDigital.xlsx
+++ b/docs/api-v3.5/matriz_api_notificacion_DocDigital.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>reports/index.html; cucumber @Notificacion_HappyPath; correo DocDigital id 89685</t>
+          <t>reports/index.html; cucumber @Notificacion_HappyPath; correo DocDigital id 89703 (JFC)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>POST 200 OK — ids 89685, 89687, 89688; correos recibidos: 89679, 89682, 89685, 89687</t>
+          <t>POST 200 OK — correos recibidos: 89703, 89705 (QA Notificacion JFC 13:54)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Captura bandeja correos; reports/index.html; cucumber suite completa</t>
+          <t>Captura bandeja correos 89703 y 89705; reports/index.html; cucumber suite 11/11</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>200 OK — id 89687; correo DocDigital 89687</t>
+          <t>200 OK — correo DocDigital 89705 (23-06-2026 13:54:17); materia QA Notificacion JFC</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>200 OK — id 89688 (23-06-2026 10:38:17)</t>
+          <t>200 OK — API QA acepta dependiente como principal (ver hallazgo H-01 en evidencias)</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">

</xml_diff>